<commit_message>
Pridėtas duomenų perkėlimas į Aerodinamikos, Svėrimo ir Koncentracijos lapus
</commit_message>
<xml_diff>
--- a/Pradiniai.xlsx
+++ b/Pradiniai.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-014 Darbuotojų failai/Tomo/Python 3.14.3/Skaiciavimai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_45EDA4434E0550A4F20679E990E356986B43F608" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0EE2247-77BE-4A5C-A8F7-E8975B5E3EA4}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_45EDA4434ED551BD12A477E990E356986B43F608" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3CE6ABA-12FC-4E33-8EE7-832101478D4A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -453,4 +453,317 @@
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
+    <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <xsd:import namespace="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="12" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="15" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="16" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Vaizdų žymės" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="993cf2ba-b7a7-49f7-97d1-76e12a88c412" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="24" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="aa0d983d-359a-438c-9953-3af1a8ac0831" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{82c4fa3c-500e-4213-91e5-1b9e2014ea63}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="aa0d983d-359a-438c-9953-3af1a8ac0831">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="21" nillable="true" ma:displayName="Bendrinama su" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="22" nillable="true" ma:displayName="Bendrinta su išsamia informacija" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Turinio tipas"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Antraštė"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAF4C073-65F7-41BE-937B-140FDF21FA3E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20BE762B-AE2C-417A-819B-FA4287787AAE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C8B0016-1DF9-4A25-A8C3-29385697207A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
O2, CO2 ir temperaturos lentele perkelta i A2
</commit_message>
<xml_diff>
--- a/Pradiniai.xlsx
+++ b/Pradiniai.xlsx
@@ -17,12 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.\1"/>
-    <numFmt numFmtId="165" formatCode="0.1"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +30,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <charset val="186"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -41,13 +37,6 @@
       <name val="Times New Roman"/>
       <charset val="186"/>
       <family val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="186"/>
-      <family val="2"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -62,27 +51,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -164,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,51 +146,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -611,7 +578,7 @@
       </c>
     </row>
     <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="8" t="n">
         <v>46063</v>
       </c>
       <c r="B6" s="2" t="n">
@@ -647,121 +614,121 @@
   </cols>
   <sheetData>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 1 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 2 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 3 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 4 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 5 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Atmosferinis slėgis P, hPa</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>Statinis slėgis ortakyje ± ΔP, hPa</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="13" t="n">
         <v>1012</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="12" t="n">
         <v>-0.25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="15" t="n"/>
+      <c r="F8" s="14" t="n"/>
+      <c r="G8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="16" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -778,61 +745,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="G5:I8"/>
+  <dimension ref="A2:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15" customWidth="1" min="7" max="8"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="1" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="5" ht="39" customHeight="1">
-      <c r="G5" s="12" t="inlineStr">
+    <row r="2" ht="43.5" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Išmatuota O2 koncentracija (%)</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Išmatuota CO2 koncentracija (%)</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Temperatūra ortakyje tor (°C)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="G6" s="17" t="n">
+    <row r="3">
+      <c r="A3" s="16" t="n">
         <v>10.02</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="B3" s="16" t="n">
         <v>4.1</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="C3" s="17" t="n">
         <v>40.2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="G7" s="17" t="n">
+    <row r="4">
+      <c r="A4" s="16" t="n">
         <v>9.98</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="B4" s="16" t="n">
         <v>3.9</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="C4" s="17" t="n">
         <v>39.8</v>
       </c>
     </row>
-    <row r="8">
-      <c r="G8" s="17" t="n">
+    <row r="5">
+      <c r="A5" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="B5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="C5" s="17" t="n">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Pakeista Pradiniai2Funkcija.py dėl diferencinių slėgių įrašymo į Paėmimas
</commit_message>
<xml_diff>
--- a/Pradiniai.xlsx
+++ b/Pradiniai.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
@@ -51,7 +56,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -81,6 +86,21 @@
       <right style="thin">
         <color auto="1"/>
       </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -138,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -146,44 +166,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -578,7 +604,7 @@
       </c>
     </row>
     <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="3" t="n">
         <v>46063</v>
       </c>
       <c r="B6" s="2" t="n">
@@ -614,121 +640,121 @@
   </cols>
   <sheetData>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 1 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 2 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 3 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 4 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 5 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Atmosferinis slėgis P, hPa</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>Statinis slėgis ortakyje ± ΔP, hPa</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="15" t="n">
         <v>1012</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="14" t="n">
         <v>-0.25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="16" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -754,52 +780,52 @@
   </cols>
   <sheetData>
     <row r="2" ht="43.5" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Išmatuota O2 koncentracija (%)</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Išmatuota CO2 koncentracija (%)</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Temperatūra ortakyje tor (°C)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="18" t="n">
         <v>10.02</v>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="18" t="n">
         <v>4.1</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="19" t="n">
         <v>40.2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="18" t="n">
         <v>9.98</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="18" t="n">
         <v>3.9</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="19" t="n">
         <v>39.8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="19" t="n">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Parenkamas geriausias variantas izokinetiškumui pasiekti
</commit_message>
<xml_diff>
--- a/Pradiniai.xlsx
+++ b/Pradiniai.xlsx
@@ -22,13 +22,18 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -47,12 +52,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -134,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -142,53 +162,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -559,13 +582,13 @@
   <dimension ref="A5:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="25" customWidth="1" style="13" min="1" max="1"/>
-    <col width="40" customWidth="1" style="13" min="2" max="2"/>
-    <col width="60" customWidth="1" style="13" min="3" max="3"/>
-    <col width="20" customWidth="1" style="13" min="4" max="4"/>
+    <col width="25" customWidth="1" style="11" min="1" max="1"/>
+    <col width="40" customWidth="1" style="11" min="2" max="2"/>
+    <col width="60" customWidth="1" style="11" min="3" max="3"/>
+    <col width="20" customWidth="1" style="11" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="5" ht="40" customHeight="1" s="13">
+    <row r="5" ht="40" customHeight="1" s="11">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Matavimo data</t>
@@ -587,8 +610,8 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1" s="13">
-      <c r="A6" s="14" t="n">
+    <row r="6" ht="50" customHeight="1" s="11">
+      <c r="A6" s="3" t="n">
         <v>46063</v>
       </c>
       <c r="B6" s="2" t="n">
@@ -619,107 +642,107 @@
   <dimension ref="A5:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15" customWidth="1" style="13" min="1" max="2"/>
-    <col width="15" customWidth="1" style="13" min="2" max="2"/>
-    <col width="18" customWidth="1" style="13" min="3" max="4"/>
-    <col width="18" customWidth="1" style="13" min="4" max="4"/>
+    <col width="15" customWidth="1" style="11" min="1" max="2"/>
+    <col width="15" customWidth="1" style="11" min="2" max="2"/>
+    <col width="18" customWidth="1" style="11" min="3" max="4"/>
+    <col width="18" customWidth="1" style="11" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="5" ht="58" customHeight="1" s="13">
-      <c r="A5" s="15" t="inlineStr">
+    <row r="5" ht="58" customHeight="1" s="11">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 1 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Išmatuotas diferencinis slėgis taškuose 2 linija, Pdi, hPa</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Atmosferinis slėgis P, hPa</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Statinis slėgis ortakyje ± ΔP, hPa</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="17" t="n">
         <v>0.73</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <v>0.61</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="18" t="n">
         <v>1012</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="17" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="17" t="n">
         <v>0.87</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="17" t="n">
         <v>0.76</v>
       </c>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="17" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="17" t="n">
         <v>0.78</v>
       </c>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="17" t="n">
         <v>0.92</v>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <v>0.87</v>
       </c>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="17" t="n">
         <v>0.86</v>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="17" t="n">
         <v>0.82</v>
       </c>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="17" t="n">
         <v>0.77</v>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="17" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n">
+      <c r="A12" s="17" t="n">
         <v>0.7</v>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="17" t="n">
         <v>0.75</v>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
+      <c r="C12" s="20" t="n"/>
+      <c r="D12" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -739,54 +762,54 @@
   <dimension ref="B5:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="22" customWidth="1" style="13" min="2" max="6"/>
-    <col width="22" customWidth="1" style="13" min="3" max="3"/>
-    <col width="22" customWidth="1" style="13" min="4" max="4"/>
-    <col width="22" customWidth="1" style="13" min="5" max="5"/>
-    <col width="22" customWidth="1" style="13" min="6" max="6"/>
+    <col width="22" customWidth="1" style="11" min="2" max="6"/>
+    <col width="22" customWidth="1" style="11" min="3" max="3"/>
+    <col width="22" customWidth="1" style="11" min="4" max="4"/>
+    <col width="22" customWidth="1" style="11" min="5" max="5"/>
+    <col width="22" customWidth="1" style="11" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="5" ht="29" customHeight="1" s="13">
-      <c r="B5" s="15" t="inlineStr">
+    <row r="5" ht="29" customHeight="1" s="11">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Ėminių ėmimo laikas t, min.</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Paėmimo greitis, l/min</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Išretėjimas, -hPa</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Temperatūra prie aspiratoriaus, Vtr oC</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>Vandens kondensato masė m H2O, kg</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="21" t="n">
         <v>27.2</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="21" t="n">
         <v>12.7</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="22" t="n">
         <v>0.015</v>
       </c>
     </row>
@@ -804,377 +827,377 @@
   <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="18" customWidth="1" style="13" min="1" max="12"/>
-    <col width="18" customWidth="1" style="13" min="2" max="2"/>
-    <col width="18" customWidth="1" style="13" min="3" max="3"/>
-    <col width="18" customWidth="1" style="13" min="4" max="4"/>
-    <col width="18" customWidth="1" style="13" min="5" max="5"/>
-    <col width="18" customWidth="1" style="13" min="6" max="6"/>
-    <col width="18" customWidth="1" style="13" min="7" max="7"/>
-    <col width="18" customWidth="1" style="13" min="8" max="8"/>
-    <col width="18" customWidth="1" style="13" min="9" max="9"/>
-    <col width="18" customWidth="1" style="13" min="10" max="10"/>
-    <col width="18" customWidth="1" style="13" min="11" max="11"/>
-    <col width="18" customWidth="1" style="13" min="12" max="12"/>
+    <col width="18" customWidth="1" style="11" min="1" max="12"/>
+    <col width="18" customWidth="1" style="11" min="2" max="2"/>
+    <col width="18" customWidth="1" style="11" min="3" max="3"/>
+    <col width="18" customWidth="1" style="11" min="4" max="4"/>
+    <col width="18" customWidth="1" style="11" min="5" max="5"/>
+    <col width="18" customWidth="1" style="11" min="6" max="6"/>
+    <col width="18" customWidth="1" style="11" min="7" max="7"/>
+    <col width="18" customWidth="1" style="11" min="8" max="8"/>
+    <col width="18" customWidth="1" style="11" min="9" max="9"/>
+    <col width="18" customWidth="1" style="11" min="10" max="10"/>
+    <col width="18" customWidth="1" style="11" min="11" max="11"/>
+    <col width="18" customWidth="1" style="11" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1"/>
-    <row r="2" ht="29" customHeight="1" s="13">
-      <c r="A2" s="15" t="inlineStr">
+    <row r="2" ht="29" customHeight="1" s="11">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Išmatuota O2 koncentracija (%)</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Išmatuota CO2 koncentracija (%)</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr">
         <is>
           <t>Temperatūra ortakyje tor (°C)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="17" t="n">
         <v>7.92</v>
       </c>
-      <c r="B3" s="16" t="n">
+      <c r="B3" s="17" t="n">
         <v>7.41</v>
       </c>
-      <c r="C3" s="20" t="n">
+      <c r="C3" s="21" t="n">
         <v>63.1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="17" t="n">
         <v>7.94</v>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>7.4</v>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="21" t="n">
         <v>62.7</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <v>7.96</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>7.39</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="21" t="n">
         <v>63.3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>1 filtras</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>1 linija</t>
         </is>
       </c>
-      <c r="G8" s="23" t="inlineStr">
+      <c r="G8" s="24" t="inlineStr">
         <is>
           <t>2 linija</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="43.5" customHeight="1" s="13">
-      <c r="A9" s="15" t="inlineStr">
+    <row r="9" ht="43.5" customHeight="1" s="11">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Slėgis prieš rotametrą ΔPr (±hPa)</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Antgalio diametras da (mm)</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Siurbimo laikas t (min)</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Siurbimo greitis Vo (l/min)</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Siurbiamų dujų temperatūra prieš rotametrą tr (°C)</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Slėgis prieš rotametrą ΔPr (±hPa)</t>
         </is>
       </c>
-      <c r="H9" s="15" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>Antgalio diametras da (mm)</t>
         </is>
       </c>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>Siurbimo laikas t (min)</t>
         </is>
       </c>
-      <c r="J9" s="15" t="inlineStr">
+      <c r="J9" s="16" t="inlineStr">
         <is>
           <t>Siurbimo greitis Vo (l/min)</t>
         </is>
       </c>
-      <c r="K9" s="15" t="inlineStr">
+      <c r="K9" s="16" t="inlineStr">
         <is>
           <t>Siurbiamų dujų temperatūra prieš rotametrą tr (°C)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="21" t="n">
         <v>58.6</v>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G10" s="21" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="H10" s="21">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="I10" s="18">
+        <f>C10</f>
+        <v/>
+      </c>
+      <c r="J10" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="K10" s="21" t="n">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G11" s="21" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="H11" s="21">
+        <f>B11</f>
+        <v/>
+      </c>
+      <c r="I11" s="18">
+        <f>C11</f>
+        <v/>
+      </c>
+      <c r="J11" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="K11" s="21" t="n">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="G12" s="21" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="H12" s="21">
+        <f>B12</f>
+        <v/>
+      </c>
+      <c r="I12" s="18">
+        <f>C12</f>
+        <v/>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="K12" s="21" t="n">
+        <v>13.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="H13" s="21">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="I13" s="18">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="K13" s="21" t="n">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="G14" s="21" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="H14" s="21">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="I14" s="18">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="K14" s="21" t="n">
+        <v>13.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G15" s="21" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="H15" s="21">
+        <f>B15</f>
+        <v/>
+      </c>
+      <c r="I15" s="18">
+        <f>C15</f>
+        <v/>
+      </c>
+      <c r="J15" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="K15" s="21" t="n">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" s="21" t="n">
         <v>13.4</v>
       </c>
-      <c r="G10" s="20" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="H10" s="20">
-        <f>B10</f>
-        <v/>
-      </c>
-      <c r="I10" s="17">
-        <f>C10</f>
-        <v/>
-      </c>
-      <c r="J10" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="K10" s="20" t="n">
-        <v>13.7</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="n">
-        <v>72.40000000000001</v>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="G11" s="20" t="n">
-        <v>67.59999999999999</v>
-      </c>
-      <c r="H11" s="20">
-        <f>B11</f>
-        <v/>
-      </c>
-      <c r="I11" s="17">
-        <f>C11</f>
-        <v/>
-      </c>
-      <c r="J11" s="17" t="n">
+      <c r="G16" s="21" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="H16" s="21">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="I16" s="18">
+        <f>C16</f>
+        <v/>
+      </c>
+      <c r="J16" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="K11" s="20" t="n">
-        <v>13.8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="n">
-        <v>72.7</v>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="G12" s="20" t="n">
-        <v>67.90000000000001</v>
-      </c>
-      <c r="H12" s="20">
-        <f>B12</f>
-        <v/>
-      </c>
-      <c r="I12" s="17">
-        <f>C12</f>
-        <v/>
-      </c>
-      <c r="J12" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="K12" s="20" t="n">
-        <v>13.8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="n">
-        <v>73.90000000000001</v>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="E13" s="20" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="G13" s="20" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="H13" s="20">
-        <f>B13</f>
-        <v/>
-      </c>
-      <c r="I13" s="17">
-        <f>C13</f>
-        <v/>
-      </c>
-      <c r="J13" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="K13" s="20" t="n">
-        <v>13.7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="n">
-        <v>75.09999999999999</v>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C14" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="E14" s="20" t="n">
-        <v>13.1</v>
-      </c>
-      <c r="G14" s="20" t="n">
-        <v>69.8</v>
-      </c>
-      <c r="H14" s="20">
-        <f>B14</f>
-        <v/>
-      </c>
-      <c r="I14" s="17">
-        <f>C14</f>
-        <v/>
-      </c>
-      <c r="J14" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="K14" s="20" t="n">
-        <v>13.7</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C15" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="E15" s="20" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G15" s="20" t="n">
-        <v>70.40000000000001</v>
-      </c>
-      <c r="H15" s="20">
-        <f>B15</f>
-        <v/>
-      </c>
-      <c r="I15" s="17">
-        <f>C15</f>
-        <v/>
-      </c>
-      <c r="J15" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="K15" s="20" t="n">
-        <v>13.6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="G16" s="20" t="n">
-        <v>70.7</v>
-      </c>
-      <c r="H16" s="20">
-        <f>B16</f>
-        <v/>
-      </c>
-      <c r="I16" s="17">
-        <f>C16</f>
-        <v/>
-      </c>
-      <c r="J16" s="17" t="n">
-        <v>11</v>
-      </c>
-      <c r="K16" s="20" t="n">
+      <c r="K16" s="21" t="n">
         <v>13.7</v>
       </c>
     </row>

</xml_diff>